<commit_message>
fix BBGN TL HRC2 máy đúc
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/BBGN_ThepLong.xlsx
+++ b/dataproduct.api/wwwroot/templates/BBGN_ThepLong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258008C9-4019-4E21-8176-42E201F5C409}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6557FB7-B4F2-4B29-BE1E-3CEA3CAF1E11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
@@ -25,9 +25,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>BM.16/QT.05.10</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t xml:space="preserve">        BIÊN BẢN GIAO NHẬN THÉP LỎNG</t>
+  </si>
+  <si>
+    <t>TT</t>
+  </si>
+  <si>
+    <t>Máy đúc</t>
+  </si>
+  <si>
+    <t>Mẻ</t>
+  </si>
+  <si>
+    <t>Mác thép</t>
+  </si>
+  <si>
+    <t>Thùng số</t>
+  </si>
+  <si>
+    <t>Thời gian</t>
+  </si>
+  <si>
+    <t>KL thùng &amp; thép lỏng vào bệ xoay ( tấn) - lần 1</t>
+  </si>
+  <si>
+    <t>KL thùng ( tấn) - lần 2</t>
+  </si>
+  <si>
+    <t>KL thùng thép lần 3 (tấn) (nếu có)</t>
+  </si>
+  <si>
+    <t>KL thép lỏng (tấn)</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tinh Luyện, Lên Thẳng </t>
+  </si>
+  <si>
+    <t>Phân loại</t>
+  </si>
+  <si>
+    <t>BM.28/QT.05.15</t>
   </si>
   <si>
     <r>
@@ -49,50 +91,11 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve"> 01/09/2023 </t>
+      <t xml:space="preserve"> 12/06/2026 </t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">        BIÊN BẢN GIAO NHẬN THÉP LỎNG</t>
-  </si>
-  <si>
-    <t>TT</t>
-  </si>
-  <si>
-    <t>Máy đúc</t>
-  </si>
-  <si>
-    <t>Mẻ</t>
-  </si>
-  <si>
-    <t>Mác thép</t>
-  </si>
-  <si>
-    <t>Thùng số</t>
-  </si>
-  <si>
-    <t>Thời gian</t>
-  </si>
-  <si>
-    <t>KL thùng &amp; thép lỏng vào bệ xoay ( tấn) - lần 1</t>
-  </si>
-  <si>
-    <t>KL thùng ( tấn) - lần 2</t>
-  </si>
-  <si>
-    <t>KL thùng thép lần 3 (tấn) (nếu có)</t>
-  </si>
-  <si>
-    <t>KL thép lỏng (tấn)</t>
-  </si>
-  <si>
-    <t>Ghi chú</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tinh Luyện, Lên Thẳng </t>
-  </si>
-  <si>
-    <t>Phân loại</t>
+    <t>Lần sửa đổi: 01</t>
   </si>
 </sst>
 </file>
@@ -197,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -224,6 +227,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -753,7 +759,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="M1" s="1"/>
     </row>
@@ -770,7 +776,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="M2" s="1"/>
     </row>
@@ -785,8 +791,10 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
+      <c r="K3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" s="11"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -797,7 +805,7 @@
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="7" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -823,48 +831,49 @@
     </row>
     <row r="6" spans="1:13" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="E6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="G6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="I6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="J6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="K6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="L6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="M6" s="9" t="s">
         <v>13</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A5:K5"/>
+    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>